<commit_message>
Ready to start with Codex
</commit_message>
<xml_diff>
--- a/BoM.xlsx
+++ b/BoM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/db3417d0bc8e68eb/Documents/Coding/GitHub/The-Rivaler/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="75" documentId="11_F25DC773A252ABDACC10482F39D94E805ADE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF92729E-942F-48EC-AF56-54E28242B042}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="11_F25DC773A252ABDACC10482F39D94E805ADE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4D3B1C6-F451-48C3-9678-8224BFCBF421}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="36">
   <si>
     <t>Item</t>
   </si>
@@ -127,6 +127,12 @@
   </si>
   <si>
     <t>For rotating the magazine of the launcher</t>
+  </si>
+  <si>
+    <t>3V DC Motor</t>
+  </si>
+  <si>
+    <t>For spinning the launching mechanism.</t>
   </si>
 </sst>
 </file>
@@ -190,6 +196,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -455,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="57" bestFit="1" customWidth="1"/>
@@ -658,6 +668,17 @@
         <v>33</v>
       </c>
     </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C9" r:id="rId1" display="https://www.amazon.com/WWZMDiB-Adater-Module-Support-Arduino/dp/B0B779R5TZ/ref=sr_1_3?crid=O1CNAZ30MY8T&amp;dib=eyJ2IjoiMSJ9.KAiT_ubjVZEP_XTLeoPXNij7o24g5BmMNYrFGGaANH0rXndaDUPqxjQI-1zMi6QcyQRu7v8EAWnskshtsy7fZF0twWvqXwSgWXBsyfcxrXtuIFPwB0VMr3hJydMu-bmNzwGFB9x8j27biTvI_XDpM79tqwfnvSYogqe2ys-zvjJWdG55gDVKIOVWL_mpBeNuPfohXwkgR5GjNoraUIhFxPFFsahu2i3cml8HnP0Y7jg.h4y34tIFcBM1_8pPpVFApFs6nsaaRUcNQ_toU1-4l3g&amp;dib_tag=se&amp;keywords=sd+card+module+arduino&amp;qid=1783699767&amp;sprefix=sd+card+module+arduino%2Caps%2C138&amp;sr=8-3" xr:uid="{3C588B1D-CF78-4B01-B154-B7FF89E2B8F5}"/>

</xml_diff>

<commit_message>
Almost Ready to Release
</commit_message>
<xml_diff>
--- a/BoM.xlsx
+++ b/BoM.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R678629f3c3a84d94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rea50175b24e64432"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,18 +79,18 @@
     <x:t xml:space="preserve">Buttons</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Joystick</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Switches</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Active Buzzer</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">For the remote control</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Joystick</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Switches</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Active Buzzer</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Color LED</x:t>
   </x:si>
   <x:si>
@@ -107,9 +107,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">360 Servo from Sunfounder Picrawler</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">For rotating the magazine of the launcher</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">3V DC Motor</x:t>
@@ -471,44 +468,44 @@
       <x:c r="A10" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B10">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D10" t="s">
-        <x:v>23</x:v>
+      <x:c r="B10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>Remote: Quick Shoot, Rapid Fire, Take Picture, Eject SD, and wireless emergency stop.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B11">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D11" t="s">
-        <x:v>23</x:v>
+      <x:c r="D11" t="str">
+        <x:v>Remote joystick axes plus Follow Line push switch.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B12">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D12" t="s">
-        <x:v>23</x:v>
+      <x:c r="D12" t="str">
+        <x:v>Launcher arm switch on the remote.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B13">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D13" t="s">
         <x:v>26</x:v>
-      </x:c>
-      <x:c r="B13">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D13" t="s">
-        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -519,7 +516,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D14" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -551,19 +548,19 @@
       <x:c r="B17">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D17" t="s">
-        <x:v>33</x:v>
+      <x:c r="D17" t="str">
+        <x:v>360-degree positional magazine servo: homes at 0 degrees and indexes 45, 90, 135, 180, -45, -90, -135, then 0.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B18">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D18" t="s">
         <x:v>34</x:v>
-      </x:c>
-      <x:c r="B18">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D18" t="s">
-        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -575,13 +572,13 @@
       </x:c>
       <x:c r="C19"/>
       <x:c r="D19" t="str">
-        <x:v>Dedicated driver for the launcher 3V DC motor.</x:v>
+        <x:v>Dedicated driver for the launcher 3V DC motor; digital enable runs it at full speed while armed.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="R599b3ba9da7147e3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="R7efd6f7e661c44c9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="R170d2a8bd818480d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="Rfa60ff5afd24434c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>